<commit_message>
feat: ajout du frontend minimaliste
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BraimiAlbert.xlsx
+++ b/Journal-de-Travail_BraimiAlbert.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="43">
   <si>
     <t xml:space="preserve">Journal de travail</t>
   </si>
@@ -131,6 +131,27 @@
   </si>
   <si>
     <t xml:space="preserve">Création du projet avec Avalonia </t>
+  </si>
+  <si>
+    <t xml:space="preserve">J’ai eu plusieurs erreurs de version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résolution d’erreurs par rapport à Avalonia + Scottplot et dotnet8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Installation du serveur de language roslyn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en place de l’importation des json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realisation du frontend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentation + Implémentation minimale (graphes, toggle, labels)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remplissage du jdt</t>
   </si>
 </sst>
 </file>
@@ -303,7 +324,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -483,6 +504,10 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -942,7 +967,7 @@
       <c r="B3" s="9"/>
       <c r="C3" s="13" t="str">
         <f aca="false">QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>9 heures 0 minutes</v>
+        <v>12 heures 0 minutes</v>
       </c>
       <c r="D3" s="14"/>
       <c r="E3" s="15"/>
@@ -957,15 +982,15 @@
       <c r="B4" s="11"/>
       <c r="C4" s="14" t="n">
         <f aca="false">SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="D4" s="14" t="n">
         <f aca="false">SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>360</v>
+        <v>480</v>
       </c>
       <c r="E4" s="18" t="n">
         <f aca="false">SUM(C4:D4)</f>
-        <v>540</v>
+        <v>720</v>
       </c>
       <c r="F4" s="16"/>
       <c r="G4" s="19"/>
@@ -1362,78 +1387,132 @@
       <c r="F20" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="G20" s="39"/>
+      <c r="G20" s="39" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34" t="str">
+      <c r="A21" s="45" t="n">
         <f aca="false">IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="40"/>
+        <v>38</v>
+      </c>
+      <c r="B21" s="40" t="n">
+        <v>46279</v>
+      </c>
       <c r="C21" s="41"/>
-      <c r="D21" s="42"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="32"/>
+      <c r="D21" s="42" t="n">
+        <v>15</v>
+      </c>
+      <c r="E21" s="43" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="32" t="s">
+        <v>17</v>
+      </c>
       <c r="G21" s="44"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34" t="str">
+      <c r="A22" s="45" t="n">
         <f aca="false">IF(ISBLANK(B22),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B22))</f>
-        <v/>
-      </c>
-      <c r="B22" s="35"/>
+        <v>38</v>
+      </c>
+      <c r="B22" s="35" t="n">
+        <v>46279</v>
+      </c>
       <c r="C22" s="36"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="32"/>
+      <c r="D22" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="E22" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" s="32" t="s">
+        <v>37</v>
+      </c>
       <c r="G22" s="39"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34" t="str">
+      <c r="A23" s="45" t="n">
         <f aca="false">IF(ISBLANK(B23),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B23))</f>
-        <v/>
-      </c>
-      <c r="B23" s="40"/>
+        <v>38</v>
+      </c>
+      <c r="B23" s="40" t="n">
+        <v>46279</v>
+      </c>
       <c r="C23" s="41"/>
-      <c r="D23" s="42"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="32"/>
+      <c r="D23" s="42" t="n">
+        <v>20</v>
+      </c>
+      <c r="E23" s="43" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" s="32" t="s">
+        <v>38</v>
+      </c>
       <c r="G23" s="44"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34" t="str">
+      <c r="A24" s="45" t="n">
         <f aca="false">IF(ISBLANK(B24),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B24))</f>
-        <v/>
-      </c>
-      <c r="B24" s="35"/>
+        <v>38</v>
+      </c>
+      <c r="B24" s="35" t="n">
+        <v>46279</v>
+      </c>
       <c r="C24" s="36"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="32"/>
+      <c r="D24" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="E24" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" s="32" t="s">
+        <v>39</v>
+      </c>
       <c r="G24" s="39"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="34" t="str">
+      <c r="A25" s="45" t="n">
         <f aca="false">IF(ISBLANK(B25),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B25))</f>
-        <v/>
-      </c>
-      <c r="B25" s="40"/>
-      <c r="C25" s="41"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="32"/>
-      <c r="G25" s="44"/>
+        <v>38</v>
+      </c>
+      <c r="B25" s="40" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C25" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="42" t="n">
+        <v>30</v>
+      </c>
+      <c r="E25" s="43" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="G25" s="44" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="34" t="str">
+      <c r="A26" s="45" t="n">
         <f aca="false">IF(ISBLANK(B26),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B26))</f>
-        <v/>
-      </c>
-      <c r="B26" s="35"/>
+        <v>38</v>
+      </c>
+      <c r="B26" s="35" t="n">
+        <v>46279</v>
+      </c>
       <c r="C26" s="36"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="32"/>
+      <c r="D26" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26" s="32" t="s">
+        <v>42</v>
+      </c>
       <c r="G26" s="39"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1457,7 +1536,7 @@
       <c r="C28" s="36"/>
       <c r="D28" s="37"/>
       <c r="E28" s="38"/>
-      <c r="F28" s="45"/>
+      <c r="F28" s="46"/>
       <c r="G28" s="39"/>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1469,7 +1548,7 @@
       <c r="C29" s="41"/>
       <c r="D29" s="42"/>
       <c r="E29" s="43"/>
-      <c r="F29" s="45"/>
+      <c r="F29" s="46"/>
       <c r="G29" s="44"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1493,7 +1572,7 @@
       <c r="C31" s="41"/>
       <c r="D31" s="42"/>
       <c r="E31" s="43"/>
-      <c r="F31" s="45"/>
+      <c r="F31" s="46"/>
       <c r="G31" s="44"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1517,7 +1596,7 @@
       <c r="C33" s="41"/>
       <c r="D33" s="42"/>
       <c r="E33" s="43"/>
-      <c r="F33" s="45"/>
+      <c r="F33" s="46"/>
       <c r="G33" s="44"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1529,7 +1608,7 @@
       <c r="C34" s="36"/>
       <c r="D34" s="37"/>
       <c r="E34" s="38"/>
-      <c r="F34" s="45"/>
+      <c r="F34" s="46"/>
       <c r="G34" s="39"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1553,7 +1632,7 @@
       <c r="C36" s="36"/>
       <c r="D36" s="37"/>
       <c r="E36" s="38"/>
-      <c r="F36" s="45"/>
+      <c r="F36" s="46"/>
       <c r="G36" s="39"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1565,7 +1644,7 @@
       <c r="C37" s="41"/>
       <c r="D37" s="42"/>
       <c r="E37" s="43"/>
-      <c r="F37" s="45"/>
+      <c r="F37" s="46"/>
       <c r="G37" s="44"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1577,7 +1656,7 @@
       <c r="C38" s="36"/>
       <c r="D38" s="37"/>
       <c r="E38" s="38"/>
-      <c r="F38" s="45"/>
+      <c r="F38" s="46"/>
       <c r="G38" s="39"/>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1589,7 +1668,7 @@
       <c r="C39" s="41"/>
       <c r="D39" s="42"/>
       <c r="E39" s="43"/>
-      <c r="F39" s="45"/>
+      <c r="F39" s="46"/>
       <c r="G39" s="44"/>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1601,7 +1680,7 @@
       <c r="C40" s="36"/>
       <c r="D40" s="37"/>
       <c r="E40" s="38"/>
-      <c r="F40" s="45"/>
+      <c r="F40" s="46"/>
       <c r="G40" s="39"/>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1613,7 +1692,7 @@
       <c r="C41" s="41"/>
       <c r="D41" s="42"/>
       <c r="E41" s="43"/>
-      <c r="F41" s="45"/>
+      <c r="F41" s="46"/>
       <c r="G41" s="44"/>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1625,7 +1704,7 @@
       <c r="C42" s="36"/>
       <c r="D42" s="37"/>
       <c r="E42" s="38"/>
-      <c r="F42" s="45"/>
+      <c r="F42" s="46"/>
       <c r="G42" s="39"/>
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1637,7 +1716,7 @@
       <c r="C43" s="41"/>
       <c r="D43" s="42"/>
       <c r="E43" s="43"/>
-      <c r="F43" s="45"/>
+      <c r="F43" s="46"/>
       <c r="G43" s="44"/>
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1649,7 +1728,7 @@
       <c r="C44" s="36"/>
       <c r="D44" s="37"/>
       <c r="E44" s="38"/>
-      <c r="F44" s="45"/>
+      <c r="F44" s="46"/>
       <c r="G44" s="39"/>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1661,7 +1740,7 @@
       <c r="C45" s="41"/>
       <c r="D45" s="42"/>
       <c r="E45" s="43"/>
-      <c r="F45" s="45"/>
+      <c r="F45" s="46"/>
       <c r="G45" s="44"/>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1673,7 +1752,7 @@
       <c r="C46" s="36"/>
       <c r="D46" s="37"/>
       <c r="E46" s="38"/>
-      <c r="F46" s="45"/>
+      <c r="F46" s="46"/>
       <c r="G46" s="39"/>
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1685,7 +1764,7 @@
       <c r="C47" s="41"/>
       <c r="D47" s="42"/>
       <c r="E47" s="43"/>
-      <c r="F47" s="45"/>
+      <c r="F47" s="46"/>
       <c r="G47" s="44"/>
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1697,7 +1776,7 @@
       <c r="C48" s="36"/>
       <c r="D48" s="37"/>
       <c r="E48" s="38"/>
-      <c r="F48" s="45"/>
+      <c r="F48" s="46"/>
       <c r="G48" s="39"/>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1709,7 +1788,7 @@
       <c r="C49" s="41"/>
       <c r="D49" s="42"/>
       <c r="E49" s="43"/>
-      <c r="F49" s="45"/>
+      <c r="F49" s="46"/>
       <c r="G49" s="44"/>
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1721,7 +1800,7 @@
       <c r="C50" s="36"/>
       <c r="D50" s="37"/>
       <c r="E50" s="38"/>
-      <c r="F50" s="45"/>
+      <c r="F50" s="46"/>
       <c r="G50" s="39"/>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1733,7 +1812,7 @@
       <c r="C51" s="41"/>
       <c r="D51" s="42"/>
       <c r="E51" s="43"/>
-      <c r="F51" s="45"/>
+      <c r="F51" s="46"/>
       <c r="G51" s="44"/>
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1745,7 +1824,7 @@
       <c r="C52" s="36"/>
       <c r="D52" s="37"/>
       <c r="E52" s="38"/>
-      <c r="F52" s="45"/>
+      <c r="F52" s="46"/>
       <c r="G52" s="39"/>
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1757,7 +1836,7 @@
       <c r="C53" s="41"/>
       <c r="D53" s="42"/>
       <c r="E53" s="43"/>
-      <c r="F53" s="45"/>
+      <c r="F53" s="46"/>
       <c r="G53" s="44"/>
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1769,7 +1848,7 @@
       <c r="C54" s="36"/>
       <c r="D54" s="37"/>
       <c r="E54" s="38"/>
-      <c r="F54" s="45"/>
+      <c r="F54" s="46"/>
       <c r="G54" s="39"/>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1781,7 +1860,7 @@
       <c r="C55" s="41"/>
       <c r="D55" s="42"/>
       <c r="E55" s="43"/>
-      <c r="F55" s="45"/>
+      <c r="F55" s="46"/>
       <c r="G55" s="44"/>
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore: ajout su jdt
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BraimiAlbert.xlsx
+++ b/Journal-de-Travail_BraimiAlbert.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="52">
   <si>
     <t xml:space="preserve">Journal de travail</t>
   </si>
@@ -170,6 +170,15 @@
   </si>
   <si>
     <t xml:space="preserve">Revue de l’app avec le prof</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ajout d'un merge pour les imports</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai aussi fait en sorte que scottplot ne fasse pas de liaison entre les points trop espacés pour eviter une fausse liaison entre deux imports qui auraient un expace entre deux et donc des données manquantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remplissage du jdt</t>
   </si>
 </sst>
 </file>
@@ -342,7 +351,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -530,6 +539,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -993,7 +1006,7 @@
       <c r="B3" s="10"/>
       <c r="C3" s="14" t="str">
         <f aca="false">QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>15 heures 0 minutes</v>
+        <v>18 heures 0 minutes</v>
       </c>
       <c r="D3" s="15"/>
       <c r="E3" s="16"/>
@@ -1008,15 +1021,15 @@
       <c r="B4" s="12"/>
       <c r="C4" s="15" t="n">
         <f aca="false">SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>300</v>
+        <v>420</v>
       </c>
       <c r="D4" s="15" t="n">
         <f aca="false">SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>600</v>
+        <v>660</v>
       </c>
       <c r="E4" s="19" t="n">
         <f aca="false">SUM(C4:D4)</f>
-        <v>900</v>
+        <v>1080</v>
       </c>
       <c r="F4" s="17"/>
       <c r="G4" s="20"/>
@@ -1646,11 +1659,13 @@
       <c r="G31" s="45"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="35" t="str">
+      <c r="A32" s="35" t="n">
         <f aca="false">IF(ISBLANK(B32),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B32))</f>
-        <v/>
-      </c>
-      <c r="B32" s="36"/>
+        <v>40</v>
+      </c>
+      <c r="B32" s="36" t="n">
+        <v>46293</v>
+      </c>
       <c r="C32" s="37"/>
       <c r="D32" s="38" t="n">
         <v>15</v>
@@ -1664,40 +1679,68 @@
       <c r="G32" s="40"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="35" t="str">
+      <c r="A33" s="35" t="n">
         <f aca="false">IF(ISBLANK(B33),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B33))</f>
-        <v/>
-      </c>
-      <c r="B33" s="41"/>
+        <v>41</v>
+      </c>
+      <c r="B33" s="41" t="n">
+        <v>46300</v>
+      </c>
       <c r="C33" s="42"/>
-      <c r="D33" s="43"/>
-      <c r="E33" s="44"/>
-      <c r="F33" s="46"/>
+      <c r="D33" s="43" t="n">
+        <v>15</v>
+      </c>
+      <c r="E33" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="F33" s="46" t="s">
+        <v>17</v>
+      </c>
       <c r="G33" s="45"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="35" t="str">
+      <c r="A34" s="35" t="n">
         <f aca="false">IF(ISBLANK(B34),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B34))</f>
-        <v/>
-      </c>
-      <c r="B34" s="36"/>
+        <v>41</v>
+      </c>
+      <c r="B34" s="36" t="n">
+        <v>46300</v>
+      </c>
       <c r="C34" s="37"/>
-      <c r="D34" s="38"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="46"/>
+      <c r="D34" s="38" t="n">
+        <v>15</v>
+      </c>
+      <c r="E34" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="F34" s="46" t="s">
+        <v>44</v>
+      </c>
       <c r="G34" s="40"/>
     </row>
-    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="35" t="str">
+    <row r="35" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="35" t="n">
         <f aca="false">IF(ISBLANK(B35),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B35))</f>
-        <v/>
-      </c>
-      <c r="B35" s="41"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="44"/>
-      <c r="F35" s="33"/>
-      <c r="G35" s="45"/>
+        <v>41</v>
+      </c>
+      <c r="B35" s="41" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C35" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="43" t="n">
+        <v>20</v>
+      </c>
+      <c r="E35" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="F35" s="47" t="s">
+        <v>49</v>
+      </c>
+      <c r="G35" s="47" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="35" t="str">
@@ -1706,9 +1749,15 @@
       </c>
       <c r="B36" s="36"/>
       <c r="C36" s="37"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="46"/>
+      <c r="D36" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="E36" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="F36" s="46" t="s">
+        <v>51</v>
+      </c>
       <c r="G36" s="40"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
feat(imports): ajout d'un bouton pour importer les données depuis l'api de la NOAA
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BraimiAlbert.xlsx
+++ b/Journal-de-Travail_BraimiAlbert.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="53">
   <si>
     <t xml:space="preserve">Journal de travail</t>
   </si>
@@ -179,6 +179,9 @@
   </si>
   <si>
     <t xml:space="preserve">remplissage du jdt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout bouton pour importer les données direct depuis l’api de la noaa</t>
   </si>
 </sst>
 </file>
@@ -540,7 +543,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1006,7 +1009,7 @@
       <c r="B3" s="10"/>
       <c r="C3" s="14" t="str">
         <f aca="false">QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>18 heures 0 minutes</v>
+        <v>18 heures 45 minutes</v>
       </c>
       <c r="D3" s="15"/>
       <c r="E3" s="16"/>
@@ -1025,11 +1028,11 @@
       </c>
       <c r="D4" s="15" t="n">
         <f aca="false">SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>660</v>
+        <v>705</v>
       </c>
       <c r="E4" s="19" t="n">
         <f aca="false">SUM(C4:D4)</f>
-        <v>1080</v>
+        <v>1125</v>
       </c>
       <c r="F4" s="17"/>
       <c r="G4" s="20"/>
@@ -1761,15 +1764,23 @@
       <c r="G36" s="40"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="35" t="str">
+      <c r="A37" s="35" t="n">
         <f aca="false">IF(ISBLANK(B37),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B37))</f>
-        <v/>
-      </c>
-      <c r="B37" s="41"/>
+        <v>41</v>
+      </c>
+      <c r="B37" s="41" t="n">
+        <v>46300</v>
+      </c>
       <c r="C37" s="42"/>
-      <c r="D37" s="43"/>
-      <c r="E37" s="44"/>
-      <c r="F37" s="46"/>
+      <c r="D37" s="43" t="n">
+        <v>45</v>
+      </c>
+      <c r="E37" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="F37" s="46" t="s">
+        <v>52</v>
+      </c>
       <c r="G37" s="45"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore(readme.md): ajout de plusieurs sections dont l'usage de l'ia
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BraimiAlbert.xlsx
+++ b/Journal-de-Travail_BraimiAlbert.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="55">
   <si>
     <t xml:space="preserve">Journal de travail</t>
   </si>
@@ -182,6 +182,12 @@
   </si>
   <si>
     <t xml:space="preserve">Ajout bouton pour importer les données direct depuis l’api de la noaa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rédaction du readme.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J’ai grandement agrandi le rapport mtn que j’ai une vision totalement claire de ce projet</t>
   </si>
 </sst>
 </file>
@@ -1009,7 +1015,7 @@
       <c r="B3" s="10"/>
       <c r="C3" s="14" t="str">
         <f aca="false">QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>18 heures 45 minutes</v>
+        <v>19 heures 45 minutes</v>
       </c>
       <c r="D3" s="15"/>
       <c r="E3" s="16"/>
@@ -1024,7 +1030,7 @@
       <c r="B4" s="12"/>
       <c r="C4" s="15" t="n">
         <f aca="false">SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="D4" s="15" t="n">
         <f aca="false">SUBTOTAL(9,$D$7:$D$531)</f>
@@ -1032,7 +1038,7 @@
       </c>
       <c r="E4" s="19" t="n">
         <f aca="false">SUM(C4:D4)</f>
-        <v>1125</v>
+        <v>1185</v>
       </c>
       <c r="F4" s="17"/>
       <c r="G4" s="20"/>
@@ -1746,11 +1752,13 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="35" t="str">
+      <c r="A36" s="35" t="n">
         <f aca="false">IF(ISBLANK(B36),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B36))</f>
-        <v/>
-      </c>
-      <c r="B36" s="36"/>
+        <v>41</v>
+      </c>
+      <c r="B36" s="36" t="n">
+        <v>46300</v>
+      </c>
       <c r="C36" s="37"/>
       <c r="D36" s="38" t="n">
         <v>10</v>
@@ -1784,16 +1792,26 @@
       <c r="G37" s="45"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="35" t="str">
+      <c r="A38" s="35" t="n">
         <f aca="false">IF(ISBLANK(B38),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B38))</f>
-        <v/>
-      </c>
-      <c r="B38" s="36"/>
-      <c r="C38" s="37"/>
+        <v>41</v>
+      </c>
+      <c r="B38" s="36" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C38" s="37" t="n">
+        <v>1</v>
+      </c>
       <c r="D38" s="38"/>
-      <c r="E38" s="39"/>
-      <c r="F38" s="46"/>
-      <c r="G38" s="40"/>
+      <c r="E38" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="F38" s="46" t="s">
+        <v>53</v>
+      </c>
+      <c r="G38" s="40" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="35" t="str">

</xml_diff>

<commit_message>
feat(ui): ajout d'une barre de défilement y et deplacement des légendes
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BraimiAlbert.xlsx
+++ b/Journal-de-Travail_BraimiAlbert.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="56">
   <si>
     <t xml:space="preserve">Journal de travail</t>
   </si>
@@ -188,6 +188,9 @@
   </si>
   <si>
     <t xml:space="preserve">J’ai grandement agrandi le rapport mtn que j’ai une vision totalement claire de ce projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout de todos</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1018,7 @@
       <c r="B3" s="10"/>
       <c r="C3" s="14" t="str">
         <f aca="false">QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>19 heures 45 minutes</v>
+        <v>20 heures 25 minutes</v>
       </c>
       <c r="D3" s="15"/>
       <c r="E3" s="16"/>
@@ -1034,11 +1037,11 @@
       </c>
       <c r="D4" s="15" t="n">
         <f aca="false">SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>705</v>
+        <v>745</v>
       </c>
       <c r="E4" s="19" t="n">
         <f aca="false">SUM(C4:D4)</f>
-        <v>1185</v>
+        <v>1225</v>
       </c>
       <c r="F4" s="17"/>
       <c r="G4" s="20"/>
@@ -1814,15 +1817,23 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="35" t="str">
+      <c r="A39" s="35" t="n">
         <f aca="false">IF(ISBLANK(B39),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B39))</f>
-        <v/>
-      </c>
-      <c r="B39" s="41"/>
+        <v>42</v>
+      </c>
+      <c r="B39" s="41" t="n">
+        <v>46307</v>
+      </c>
       <c r="C39" s="42"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="44"/>
-      <c r="F39" s="46"/>
+      <c r="D39" s="43" t="n">
+        <v>40</v>
+      </c>
+      <c r="E39" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="F39" s="46" t="s">
+        <v>55</v>
+      </c>
       <c r="G39" s="45"/>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore: ajout du jdt
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BraimiAlbert.xlsx
+++ b/Journal-de-Travail_BraimiAlbert.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="57">
   <si>
     <t xml:space="preserve">Journal de travail</t>
   </si>
@@ -191,6 +191,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ajout de todos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout d'une barre de défilement y et deplacement des légendes</t>
   </si>
 </sst>
 </file>
@@ -1018,7 +1021,7 @@
       <c r="B3" s="10"/>
       <c r="C3" s="14" t="str">
         <f aca="false">QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>20 heures 25 minutes</v>
+        <v>21 heures 5 minutes</v>
       </c>
       <c r="D3" s="15"/>
       <c r="E3" s="16"/>
@@ -1037,11 +1040,11 @@
       </c>
       <c r="D4" s="15" t="n">
         <f aca="false">SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>745</v>
+        <v>785</v>
       </c>
       <c r="E4" s="19" t="n">
         <f aca="false">SUM(C4:D4)</f>
-        <v>1225</v>
+        <v>1265</v>
       </c>
       <c r="F4" s="17"/>
       <c r="G4" s="20"/>
@@ -1843,9 +1846,15 @@
       </c>
       <c r="B40" s="36"/>
       <c r="C40" s="37"/>
-      <c r="D40" s="38"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="46"/>
+      <c r="D40" s="38" t="n">
+        <v>40</v>
+      </c>
+      <c r="E40" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="F40" s="46" t="s">
+        <v>56</v>
+      </c>
       <c r="G40" s="40"/>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>